<commit_message>
Update tournament data — Jun 09, 2026
</commit_message>
<xml_diff>
--- a/MIGC_Season_Dashboard.xlsx
+++ b/MIGC_Season_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevinvargas/Desktop/migc-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F80C3186-3B4A-B84A-9520-3A7908B8A5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A34BACC-06D7-764E-81A9-F020DB27E058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16780" yWindow="600" windowWidth="16820" windowHeight="19160" activeTab="3" xr2:uid="{BBF77493-EF1A-3942-9440-E7AC2E03DB26}"/>
   </bookViews>
@@ -592,7 +592,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -676,7 +676,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11026,7 +11025,7 @@
         <f>_xlfn.XLOOKUP(C47,Players!B:B,Players!A:A)</f>
         <v>15</v>
       </c>
-      <c r="C47" s="33" t="s">
+      <c r="C47" s="17" t="s">
         <v>11</v>
       </c>
       <c r="D47" t="s">
@@ -11047,7 +11046,7 @@
         <f>_xlfn.XLOOKUP(C48,Players!B:B,Players!A:A)</f>
         <v>13</v>
       </c>
-      <c r="C48" s="33" t="s">
+      <c r="C48" s="17" t="s">
         <v>14</v>
       </c>
       <c r="D48" t="s">
@@ -11068,7 +11067,7 @@
         <f>_xlfn.XLOOKUP(C49,Players!B:B,Players!A:A)</f>
         <v>20</v>
       </c>
-      <c r="C49" s="33" t="s">
+      <c r="C49" s="17" t="s">
         <v>18</v>
       </c>
       <c r="D49" t="s">
@@ -11089,7 +11088,7 @@
         <f>_xlfn.XLOOKUP(C50,Players!B:B,Players!A:A)</f>
         <v>44</v>
       </c>
-      <c r="C50" s="33" t="s">
+      <c r="C50" s="17" t="s">
         <v>23</v>
       </c>
       <c r="D50" t="s">
@@ -11110,7 +11109,7 @@
         <f>_xlfn.XLOOKUP(C51,Players!B:B,Players!A:A)</f>
         <v>14</v>
       </c>
-      <c r="C51" s="33" t="s">
+      <c r="C51" s="17" t="s">
         <v>26</v>
       </c>
       <c r="D51" t="s">
@@ -11131,7 +11130,7 @@
         <f>_xlfn.XLOOKUP(C52,Players!B:B,Players!A:A)</f>
         <v>10</v>
       </c>
-      <c r="C52" s="33" t="s">
+      <c r="C52" s="17" t="s">
         <v>28</v>
       </c>
       <c r="D52" t="s">
@@ -11152,7 +11151,7 @@
         <f>_xlfn.XLOOKUP(C53,Players!B:B,Players!A:A)</f>
         <v>25</v>
       </c>
-      <c r="C53" s="33" t="s">
+      <c r="C53" s="17" t="s">
         <v>38</v>
       </c>
       <c r="D53" t="s">
@@ -11173,7 +11172,7 @@
         <f>_xlfn.XLOOKUP(C54,Players!B:B,Players!A:A)</f>
         <v>43</v>
       </c>
-      <c r="C54" s="33" t="s">
+      <c r="C54" s="17" t="s">
         <v>29</v>
       </c>
       <c r="D54" t="s">
@@ -11194,7 +11193,7 @@
         <f>_xlfn.XLOOKUP(C55,Players!B:B,Players!A:A)</f>
         <v>28</v>
       </c>
-      <c r="C55" s="33" t="s">
+      <c r="C55" s="17" t="s">
         <v>35</v>
       </c>
       <c r="D55" t="s">
@@ -11215,7 +11214,7 @@
         <f>_xlfn.XLOOKUP(C56,Players!B:B,Players!A:A)</f>
         <v>1</v>
       </c>
-      <c r="C56" s="33" t="s">
+      <c r="C56" s="17" t="s">
         <v>30</v>
       </c>
       <c r="D56" t="s">
@@ -11236,7 +11235,7 @@
         <f>_xlfn.XLOOKUP(C57,Players!B:B,Players!A:A)</f>
         <v>9</v>
       </c>
-      <c r="C57" s="33" t="s">
+      <c r="C57" s="17" t="s">
         <v>37</v>
       </c>
       <c r="D57" t="s">

</xml_diff>

<commit_message>
Update tournament data — Jun 10, 2026
</commit_message>
<xml_diff>
--- a/MIGC_Season_Dashboard.xlsx
+++ b/MIGC_Season_Dashboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevinvargas/Desktop/migc-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E95F9D5F-EE64-CB44-B030-DC8AC89A6634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72413F23-772B-6840-84AE-891B0645E7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16780" yWindow="600" windowWidth="16820" windowHeight="19160" activeTab="3" xr2:uid="{BBF77493-EF1A-3942-9440-E7AC2E03DB26}"/>
+    <workbookView xWindow="22760" yWindow="600" windowWidth="28440" windowHeight="26960" activeTab="3" xr2:uid="{BBF77493-EF1A-3942-9440-E7AC2E03DB26}"/>
   </bookViews>
   <sheets>
     <sheet name="Players" sheetId="2" r:id="rId1"/>

</xml_diff>